<commit_message>
Fix: case-insensitive cal_ prefix search, now finds 19 unique variables
</commit_message>
<xml_diff>
--- a/work/tst_mdl/Foc_2024b_calibration.xlsx
+++ b/work/tst_mdl/Foc_2024b_calibration.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="320" uniqueCount="61">
   <si>
     <t>CalName</t>
   </si>
@@ -133,6 +133,69 @@
   </si>
   <si>
     <t>Foc_2024b/FieldOrientedControl/SetDutyCycle/SetDuty/Default/CalcPwmShift/Constant10</t>
+  </si>
+  <si>
+    <t>cal_AdcMaxCountsHw</t>
+  </si>
+  <si>
+    <t>cal_AdcRefVoltHw</t>
+  </si>
+  <si>
+    <t>cal_OhmRShuntHw</t>
+  </si>
+  <si>
+    <t>cal_GainAmpHw</t>
+  </si>
+  <si>
+    <t>cal_AdcVoltMidHw</t>
+  </si>
+  <si>
+    <t>cal_FullScaleCur</t>
+  </si>
+  <si>
+    <t>cal_u8TiDebPhaCur</t>
+  </si>
+  <si>
+    <t>cal_s16ThresholdPhaCurImplaisible</t>
+  </si>
+  <si>
+    <t>Constant11</t>
+  </si>
+  <si>
+    <t>Constant12</t>
+  </si>
+  <si>
+    <t>Constant13</t>
+  </si>
+  <si>
+    <t>Constant7</t>
+  </si>
+  <si>
+    <t>uint8</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/GetCurrents/AdcVolToCur/Constant</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/GetCurrents/AdcVolToCur/Constant1</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/GetCurrents/AdcVolToCur/Constant11</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/GetCurrents/AdcVolToCur/Constant12</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/GetCurrents/AdcVolToCur/Constant13</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/GetCurrents/AdcVolToCur/Constant17</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/PhaseCurrentSpikeMonitor/Constant12</t>
+  </si>
+  <si>
+    <t>Foc_2024b/FieldOrientedControl/PhaseCurrentSpikeMonitor/Constant7</t>
   </si>
 </sst>
 </file>
@@ -178,10 +241,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.140625" customWidth="true"/>
+    <col min="1" max="1" width="32.42578125" customWidth="true"/>
     <col min="2" max="2" width="11.140625" customWidth="true"/>
     <col min="3" max="3" width="10.140625" customWidth="true"/>
     <col min="4" max="4" width="12.140625" customWidth="true"/>
@@ -207,95 +270,95 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>23</v>
@@ -304,91 +367,227 @@
         <v>26</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B20" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="C20" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="0" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>